<commit_message>
Adjust inspection retry schedule
</commit_message>
<xml_diff>
--- a/config/巡检配置_示例.xlsx
+++ b/config/巡检配置_示例.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -440,11 +440,7 @@
     <col width="38" customWidth="1" min="6" max="6"/>
     <col width="38" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -490,26 +486,6 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>响应时间阈值ms</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>超时时间秒</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>轮询间隔秒</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>连续失败告警次数</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
           <t>通知组</t>
         </is>
       </c>
@@ -555,19 +531,7 @@
           <t>status=200</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>默认组</t>
         </is>
@@ -614,19 +578,7 @@
           <t>status=200; code=0</t>
         </is>
       </c>
-      <c r="I3" s="2" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="L3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>默认组</t>
         </is>

</xml_diff>

<commit_message>
Use millisecond polling config
</commit_message>
<xml_diff>
--- a/config/巡检配置_示例.xlsx
+++ b/config/巡检配置_示例.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -441,6 +441,8 @@
     <col width="38" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -486,6 +488,16 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>轮询间隔ms</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>超时时间ms</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>通知组</t>
         </is>
       </c>
@@ -531,7 +543,13 @@
           <t>status=200</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>默认组</t>
         </is>
@@ -578,7 +596,13 @@
           <t>status=200; code=0</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>默认组</t>
         </is>

</xml_diff>

<commit_message>
Use second-based polling interval
</commit_message>
<xml_diff>
--- a/config/巡检配置_示例.xlsx
+++ b/config/巡检配置_示例.xlsx
@@ -488,7 +488,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>轮询间隔ms</t>
+          <t>轮询间隔秒</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>3600000</v>
+        <v>3600</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>5000</v>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="I3" s="2" t="n">
-        <v>3600000</v>
+        <v>3600</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>5000</v>

</xml_diff>

<commit_message>
Add abnormal recovery polling interval
</commit_message>
<xml_diff>
--- a/config/巡检配置_示例.xlsx
+++ b/config/巡检配置_示例.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -441,8 +441,9 @@
     <col width="38" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -493,10 +494,15 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>异常后轮询间隔秒</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>超时时间ms</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>通知组</t>
         </is>
@@ -547,9 +553,12 @@
         <v>3600</v>
       </c>
       <c r="J2" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="K2" s="2" t="n">
         <v>5000</v>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>默认组</t>
         </is>
@@ -600,9 +609,12 @@
         <v>3600</v>
       </c>
       <c r="J3" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="K3" s="2" t="n">
         <v>5000</v>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>默认组</t>
         </is>

</xml_diff>